<commit_message>
minimal working release 1_0_0
</commit_message>
<xml_diff>
--- a/release_1_0_0/data/files/output/ml/catboost_leave_one_hotel_out.xlsx
+++ b/release_1_0_0/data/files/output/ml/catboost_leave_one_hotel_out.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -552,37 +552,37 @@
         <v>570.2660606060817</v>
       </c>
       <c r="D3" t="n">
-        <v>2139.799460440487</v>
+        <v>2030.734058040737</v>
       </c>
       <c r="E3" t="n">
-        <v>1569.533399834405</v>
+        <v>1460.467997434655</v>
       </c>
       <c r="F3" t="n">
-        <v>1569.533399834405</v>
+        <v>1460.467997434655</v>
       </c>
       <c r="G3" t="n">
         <v>233.321212121201</v>
       </c>
       <c r="H3" t="n">
-        <v>1353.538010907122</v>
+        <v>1216.650855985115</v>
       </c>
       <c r="I3" t="n">
-        <v>1120.216798785921</v>
+        <v>983.3296438639144</v>
       </c>
       <c r="J3" t="n">
-        <v>1120.216798785921</v>
+        <v>983.3296438639144</v>
       </c>
       <c r="K3" t="n">
         <v>248.7434418642236</v>
       </c>
       <c r="L3" t="n">
-        <v>1077.710273972323</v>
+        <v>1099.371092419906</v>
       </c>
       <c r="M3" t="n">
-        <v>828.9668321080995</v>
+        <v>850.6276505556826</v>
       </c>
       <c r="N3" t="n">
-        <v>828.9668321080995</v>
+        <v>850.6276505556826</v>
       </c>
     </row>
     <row r="4">
@@ -600,91 +600,91 @@
         <v>17096.63041667935</v>
       </c>
       <c r="D4" t="n">
-        <v>1829.67057197806</v>
+        <v>1873.840269506757</v>
       </c>
       <c r="E4" t="n">
-        <v>-15266.95984470129</v>
+        <v>-15222.7901471726</v>
       </c>
       <c r="F4" t="n">
-        <v>15266.95984470129</v>
+        <v>15222.7901471726</v>
       </c>
       <c r="G4" t="n">
         <v>9167.626249997114</v>
       </c>
       <c r="H4" t="n">
-        <v>1102.672115031578</v>
+        <v>1140.892289621151</v>
       </c>
       <c r="I4" t="n">
-        <v>-8064.954134965536</v>
+        <v>-8026.733960375964</v>
       </c>
       <c r="J4" t="n">
-        <v>8064.954134965536</v>
+        <v>8026.733960375964</v>
       </c>
       <c r="K4" t="n">
         <v>8864.534661573482</v>
       </c>
       <c r="L4" t="n">
-        <v>957.8236729863846</v>
+        <v>1051.371151573171</v>
       </c>
       <c r="M4" t="n">
-        <v>-7906.710988587097</v>
+        <v>-7813.163510000311</v>
       </c>
       <c r="N4" t="n">
-        <v>7906.710988587097</v>
+        <v>7813.163510000311</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>H5586</t>
+          <t>H6188</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>connected</t>
+          <t>liberty</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1438.426056822751</v>
       </c>
       <c r="D5" t="n">
-        <v>1449.850896213255</v>
+        <v>1434.927763029601</v>
       </c>
       <c r="E5" t="n">
-        <v>1449.850896213255</v>
+        <v>-3.498293793149514</v>
       </c>
       <c r="F5" t="n">
-        <v>1449.850896213255</v>
+        <v>3.498293793149514</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>750.5261190476397</v>
       </c>
       <c r="H5" t="n">
-        <v>944.6029835070754</v>
+        <v>849.2573032979535</v>
       </c>
       <c r="I5" t="n">
-        <v>944.6029835070754</v>
+        <v>98.73118425031385</v>
       </c>
       <c r="J5" t="n">
-        <v>944.6029835070754</v>
+        <v>98.73118425031385</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>795.1738730737154</v>
       </c>
       <c r="L5" t="n">
-        <v>810.6124748564513</v>
+        <v>688.3953081646137</v>
       </c>
       <c r="M5" t="n">
-        <v>810.6124748564513</v>
+        <v>-106.7785649091018</v>
       </c>
       <c r="N5" t="n">
-        <v>810.6124748564513</v>
+        <v>106.7785649091018</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>H6188</t>
+          <t>HB5I0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -693,136 +693,88 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1438.426056822751</v>
+        <v>1766.508730769235</v>
       </c>
       <c r="D6" t="n">
-        <v>1353.367878079128</v>
+        <v>1230.803738908821</v>
       </c>
       <c r="E6" t="n">
-        <v>-85.0581787436231</v>
+        <v>-535.7049918604134</v>
       </c>
       <c r="F6" t="n">
-        <v>85.0581787436231</v>
+        <v>535.7049918604134</v>
       </c>
       <c r="G6" t="n">
-        <v>750.5261190476397</v>
+        <v>974.3293076923151</v>
       </c>
       <c r="H6" t="n">
-        <v>885.0787834902281</v>
+        <v>606.9296369610985</v>
       </c>
       <c r="I6" t="n">
-        <v>134.5526644425885</v>
+        <v>-367.3996707312166</v>
       </c>
       <c r="J6" t="n">
-        <v>134.5526644425885</v>
+        <v>367.3996707312166</v>
       </c>
       <c r="K6" t="n">
-        <v>795.1738730737154</v>
+        <v>815.1594794547862</v>
       </c>
       <c r="L6" t="n">
-        <v>715.0201214757515</v>
+        <v>681.280517578125</v>
       </c>
       <c r="M6" t="n">
-        <v>-80.15375159796395</v>
+        <v>-133.8789618766612</v>
       </c>
       <c r="N6" t="n">
-        <v>80.15375159796395</v>
+        <v>133.8789618766612</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HB5I0</t>
+          <t>HB6A3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>liberty</t>
+          <t>simply</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1766.508730769235</v>
+        <v>1085.428421052641</v>
       </c>
       <c r="D7" t="n">
-        <v>1120.934650796655</v>
+        <v>1189.826043819528</v>
       </c>
       <c r="E7" t="n">
-        <v>-645.5740799725793</v>
+        <v>104.397622766887</v>
       </c>
       <c r="F7" t="n">
-        <v>645.5740799725793</v>
+        <v>104.397622766887</v>
       </c>
       <c r="G7" t="n">
-        <v>974.3293076923151</v>
+        <v>522.3989473684123</v>
       </c>
       <c r="H7" t="n">
-        <v>591.3020328753303</v>
+        <v>626.7920505406692</v>
       </c>
       <c r="I7" t="n">
-        <v>-383.0272748169848</v>
+        <v>104.3931031722568</v>
       </c>
       <c r="J7" t="n">
-        <v>383.0272748169848</v>
+        <v>104.3931031722568</v>
       </c>
       <c r="K7" t="n">
-        <v>815.1594794547862</v>
+        <v>607.1911078395337</v>
       </c>
       <c r="L7" t="n">
-        <v>645.5327272740063</v>
+        <v>662.7398369138109</v>
       </c>
       <c r="M7" t="n">
-        <v>-169.6267521807798</v>
+        <v>55.54872907427716</v>
       </c>
       <c r="N7" t="n">
-        <v>169.6267521807798</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>HB6A3</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>simply</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>1085.428421052641</v>
-      </c>
-      <c r="D8" t="n">
-        <v>876.1663440967693</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-209.2620769558714</v>
-      </c>
-      <c r="F8" t="n">
-        <v>209.2620769558714</v>
-      </c>
-      <c r="G8" t="n">
-        <v>522.3989473684123</v>
-      </c>
-      <c r="H8" t="n">
-        <v>626.7920505406692</v>
-      </c>
-      <c r="I8" t="n">
-        <v>104.3931031722568</v>
-      </c>
-      <c r="J8" t="n">
-        <v>104.3931031722568</v>
-      </c>
-      <c r="K8" t="n">
-        <v>607.1911078395337</v>
-      </c>
-      <c r="L8" t="n">
-        <v>166.4348787226038</v>
-      </c>
-      <c r="M8" t="n">
-        <v>-440.7562291169299</v>
-      </c>
-      <c r="N8" t="n">
-        <v>440.7562291169299</v>
+        <v>55.54872907427716</v>
       </c>
     </row>
   </sheetData>
@@ -891,16 +843,16 @@
         <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>2844.734449953546</v>
+        <v>2793.065201286394</v>
       </c>
       <c r="E2" t="n">
-        <v>5838.116040299871</v>
+        <v>5818.695703090997</v>
       </c>
       <c r="F2" t="n">
-        <v>74.37947996406562</v>
+        <v>67.55707022560712</v>
       </c>
       <c r="G2" t="n">
-        <v>-1785.795315867416</v>
+        <v>-1710.361493806794</v>
       </c>
     </row>
     <row r="3">
@@ -918,16 +870,16 @@
         <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>1550.070541084332</v>
+        <v>1520.047677600998</v>
       </c>
       <c r="E3" t="n">
-        <v>3102.443940798998</v>
+        <v>3081.84300694664</v>
       </c>
       <c r="F3" t="n">
-        <v>108.2954997753554</v>
+        <v>97.38505664954369</v>
       </c>
       <c r="G3" t="n">
-        <v>-891.8518125392342</v>
+        <v>-906.4895964010415</v>
       </c>
     </row>
     <row r="4">
@@ -945,16 +897,16 @@
         <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>1475.552890896289</v>
+        <v>1416.31661458942</v>
       </c>
       <c r="E4" t="n">
-        <v>3026.036849807144</v>
+        <v>2989.345871715312</v>
       </c>
       <c r="F4" t="n">
-        <v>88.4314108405286</v>
+        <v>78.96054807104936</v>
       </c>
       <c r="G4" t="n">
-        <v>-980.8036009559304</v>
+        <v>-884.7751102066013</v>
       </c>
     </row>
   </sheetData>

</xml_diff>